<commit_message>
Preisliste: Notweg auf den Stand der Datenbank gebracht
</commit_message>
<xml_diff>
--- a/Angebotsdaten.xlsx
+++ b/Angebotsdaten.xlsx
@@ -28573,7 +28573,7 @@
         </is>
       </c>
       <c r="F628" t="n">
-        <v>0</v>
+        <v>3680</v>
       </c>
       <c r="H628" t="inlineStr">
         <is>
@@ -30573,7 +30573,7 @@
         </is>
       </c>
       <c r="F673" t="n">
-        <v>0</v>
+        <v>3560</v>
       </c>
       <c r="H673" t="inlineStr">
         <is>
@@ -32655,7 +32655,7 @@
         </is>
       </c>
       <c r="F720" t="n">
-        <v>0</v>
+        <v>3560</v>
       </c>
       <c r="H720" t="inlineStr">
         <is>
@@ -34742,7 +34742,7 @@
         </is>
       </c>
       <c r="F767" t="n">
-        <v>0</v>
+        <v>3560</v>
       </c>
       <c r="H767" t="inlineStr">
         <is>
@@ -36865,7 +36865,7 @@
         </is>
       </c>
       <c r="F815" t="n">
-        <v>0</v>
+        <v>3560</v>
       </c>
       <c r="H815" t="inlineStr">
         <is>
@@ -40517,7 +40517,7 @@
         </is>
       </c>
       <c r="F897" t="n">
-        <v>0</v>
+        <v>4730</v>
       </c>
       <c r="H897" t="inlineStr">
         <is>
@@ -42430,7 +42430,7 @@
         </is>
       </c>
       <c r="F940" t="n">
-        <v>0</v>
+        <v>4330</v>
       </c>
       <c r="H940" t="inlineStr">
         <is>
@@ -43272,7 +43272,7 @@
         </is>
       </c>
       <c r="C960" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="D960" t="inlineStr">
         <is>
@@ -43318,7 +43318,7 @@
         </is>
       </c>
       <c r="C961" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="D961" t="inlineStr">
         <is>
@@ -43364,7 +43364,7 @@
         </is>
       </c>
       <c r="C962" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="D962" t="inlineStr">
         <is>
@@ -43410,7 +43410,7 @@
         </is>
       </c>
       <c r="C963" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="D963" t="inlineStr">
         <is>
@@ -43456,7 +43456,7 @@
         </is>
       </c>
       <c r="C964" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="D964" t="inlineStr">
         <is>
@@ -43502,7 +43502,7 @@
         </is>
       </c>
       <c r="C965" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="D965" t="inlineStr">
         <is>
@@ -43548,7 +43548,7 @@
         </is>
       </c>
       <c r="C966" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="D966" t="inlineStr">
         <is>
@@ -43594,7 +43594,7 @@
         </is>
       </c>
       <c r="C967" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="D967" t="inlineStr">
         <is>
@@ -43640,7 +43640,7 @@
         </is>
       </c>
       <c r="C968" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="D968" t="inlineStr">
         <is>
@@ -43686,7 +43686,7 @@
         </is>
       </c>
       <c r="C969" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="D969" t="inlineStr">
         <is>
@@ -43732,7 +43732,7 @@
         </is>
       </c>
       <c r="C970" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="D970" t="inlineStr">
         <is>
@@ -43778,7 +43778,7 @@
         </is>
       </c>
       <c r="C971" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="D971" t="inlineStr">
         <is>
@@ -43819,7 +43819,7 @@
         </is>
       </c>
       <c r="C972" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="D972" t="inlineStr">
         <is>
@@ -43860,7 +43860,7 @@
         </is>
       </c>
       <c r="C973" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="D973" t="inlineStr">
         <is>
@@ -43901,7 +43901,7 @@
         </is>
       </c>
       <c r="C974" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="D974" t="inlineStr">
         <is>
@@ -43942,7 +43942,7 @@
         </is>
       </c>
       <c r="C975" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="D975" t="inlineStr">
         <is>
@@ -43983,7 +43983,7 @@
         </is>
       </c>
       <c r="C976" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="D976" t="inlineStr">
         <is>
@@ -44029,7 +44029,7 @@
         </is>
       </c>
       <c r="C977" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="D977" t="inlineStr">
         <is>
@@ -44070,7 +44070,7 @@
         </is>
       </c>
       <c r="C978" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="D978" t="inlineStr">
         <is>
@@ -44111,7 +44111,7 @@
         </is>
       </c>
       <c r="C979" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="D979" t="inlineStr">
         <is>
@@ -44152,7 +44152,7 @@
         </is>
       </c>
       <c r="C980" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D980" t="inlineStr">
         <is>
@@ -44198,7 +44198,7 @@
         </is>
       </c>
       <c r="C981" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D981" t="inlineStr">
         <is>
@@ -44244,7 +44244,7 @@
         </is>
       </c>
       <c r="C982" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D982" t="inlineStr">
         <is>
@@ -44290,7 +44290,7 @@
         </is>
       </c>
       <c r="C983" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D983" t="inlineStr">
         <is>
@@ -44336,7 +44336,7 @@
         </is>
       </c>
       <c r="C984" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D984" t="inlineStr">
         <is>
@@ -44382,7 +44382,7 @@
         </is>
       </c>
       <c r="C985" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D985" t="inlineStr">
         <is>
@@ -44428,7 +44428,7 @@
         </is>
       </c>
       <c r="C986" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D986" t="inlineStr">
         <is>
@@ -44474,7 +44474,7 @@
         </is>
       </c>
       <c r="C987" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D987" t="inlineStr">
         <is>
@@ -44520,7 +44520,7 @@
         </is>
       </c>
       <c r="C988" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D988" t="inlineStr">
         <is>
@@ -44566,7 +44566,7 @@
         </is>
       </c>
       <c r="C989" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D989" t="inlineStr">
         <is>
@@ -44612,7 +44612,7 @@
         </is>
       </c>
       <c r="C990" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D990" t="inlineStr">
         <is>
@@ -44658,7 +44658,7 @@
         </is>
       </c>
       <c r="C991" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D991" t="inlineStr">
         <is>
@@ -44704,7 +44704,7 @@
         </is>
       </c>
       <c r="C992" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D992" t="inlineStr">
         <is>
@@ -44750,7 +44750,7 @@
         </is>
       </c>
       <c r="C993" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D993" t="inlineStr">
         <is>
@@ -44796,7 +44796,7 @@
         </is>
       </c>
       <c r="C994" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D994" t="inlineStr">
         <is>
@@ -44842,7 +44842,7 @@
         </is>
       </c>
       <c r="C995" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D995" t="inlineStr">
         <is>
@@ -44888,7 +44888,7 @@
         </is>
       </c>
       <c r="C996" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D996" t="inlineStr">
         <is>
@@ -44934,7 +44934,7 @@
         </is>
       </c>
       <c r="C997" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D997" t="inlineStr">
         <is>
@@ -44980,7 +44980,7 @@
         </is>
       </c>
       <c r="C998" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D998" t="inlineStr">
         <is>
@@ -45026,7 +45026,7 @@
         </is>
       </c>
       <c r="C999" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D999" t="inlineStr">
         <is>
@@ -45072,7 +45072,7 @@
         </is>
       </c>
       <c r="C1000" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1000" t="inlineStr">
         <is>
@@ -45118,7 +45118,7 @@
         </is>
       </c>
       <c r="C1001" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1001" t="inlineStr">
         <is>
@@ -45164,7 +45164,7 @@
         </is>
       </c>
       <c r="C1002" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1002" t="inlineStr">
         <is>
@@ -45210,7 +45210,7 @@
         </is>
       </c>
       <c r="C1003" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1003" t="inlineStr">
         <is>
@@ -45256,7 +45256,7 @@
         </is>
       </c>
       <c r="C1004" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1004" t="inlineStr">
         <is>
@@ -45302,7 +45302,7 @@
         </is>
       </c>
       <c r="C1005" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1005" t="inlineStr">
         <is>
@@ -45348,7 +45348,7 @@
         </is>
       </c>
       <c r="C1006" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1006" t="inlineStr">
         <is>
@@ -45394,7 +45394,7 @@
         </is>
       </c>
       <c r="C1007" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1007" t="inlineStr">
         <is>
@@ -45440,7 +45440,7 @@
         </is>
       </c>
       <c r="C1008" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1008" t="inlineStr">
         <is>
@@ -45486,7 +45486,7 @@
         </is>
       </c>
       <c r="C1009" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1009" t="inlineStr">
         <is>
@@ -45532,7 +45532,7 @@
         </is>
       </c>
       <c r="C1010" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1010" t="inlineStr">
         <is>
@@ -45578,7 +45578,7 @@
         </is>
       </c>
       <c r="C1011" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1011" t="inlineStr">
         <is>
@@ -45624,7 +45624,7 @@
         </is>
       </c>
       <c r="C1012" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1012" t="inlineStr">
         <is>
@@ -45670,7 +45670,7 @@
         </is>
       </c>
       <c r="C1013" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1013" t="inlineStr">
         <is>
@@ -45679,7 +45679,7 @@
       </c>
       <c r="E1013" t="inlineStr">
         <is>
-          <t>Ausgklappbare 2.US</t>
+          <t>Ausklappbare 2.US</t>
         </is>
       </c>
       <c r="F1013" t="n">
@@ -45716,7 +45716,7 @@
         </is>
       </c>
       <c r="C1014" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1014" t="inlineStr">
         <is>
@@ -45762,7 +45762,7 @@
         </is>
       </c>
       <c r="C1015" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1015" t="inlineStr">
         <is>
@@ -45808,7 +45808,7 @@
         </is>
       </c>
       <c r="C1016" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1016" t="inlineStr">
         <is>
@@ -45854,7 +45854,7 @@
         </is>
       </c>
       <c r="C1017" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1017" t="inlineStr">
         <is>
@@ -45900,7 +45900,7 @@
         </is>
       </c>
       <c r="C1018" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1018" t="inlineStr">
         <is>
@@ -45946,7 +45946,7 @@
         </is>
       </c>
       <c r="C1019" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1019" t="inlineStr">
         <is>
@@ -45992,7 +45992,7 @@
         </is>
       </c>
       <c r="C1020" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="D1020" t="inlineStr">
         <is>
@@ -46038,7 +46038,7 @@
         </is>
       </c>
       <c r="C1021" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="D1021" t="inlineStr">
         <is>
@@ -46084,7 +46084,7 @@
         </is>
       </c>
       <c r="C1022" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="D1022" t="inlineStr">
         <is>
@@ -46130,7 +46130,7 @@
         </is>
       </c>
       <c r="C1023" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="D1023" t="inlineStr">
         <is>
@@ -46176,7 +46176,7 @@
         </is>
       </c>
       <c r="C1024" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="D1024" t="inlineStr">
         <is>
@@ -46222,7 +46222,7 @@
         </is>
       </c>
       <c r="C1025" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="D1025" t="inlineStr">
         <is>
@@ -46268,7 +46268,7 @@
         </is>
       </c>
       <c r="C1026" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="D1026" t="inlineStr">
         <is>
@@ -46314,7 +46314,7 @@
         </is>
       </c>
       <c r="C1027" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="D1027" t="inlineStr">
         <is>
@@ -46360,7 +46360,7 @@
         </is>
       </c>
       <c r="C1028" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="D1028" t="inlineStr">
         <is>
@@ -46866,7 +46866,7 @@
         </is>
       </c>
       <c r="C1039" t="n">
-        <v>0</v>
+        <v>8800</v>
       </c>
       <c r="D1039" t="inlineStr">
         <is>
@@ -46875,7 +46875,7 @@
       </c>
       <c r="E1039" t="inlineStr">
         <is>
-          <t>1/1 Seite</t>
+          <t>1/1 Seite 4c</t>
         </is>
       </c>
       <c r="F1039" t="n">
@@ -46912,7 +46912,7 @@
         </is>
       </c>
       <c r="C1040" t="n">
-        <v>0</v>
+        <v>8800</v>
       </c>
       <c r="D1040" t="inlineStr">
         <is>
@@ -46921,7 +46921,7 @@
       </c>
       <c r="E1040" t="inlineStr">
         <is>
-          <t>1/2 Seite</t>
+          <t>1/2 Seite 4c</t>
         </is>
       </c>
       <c r="F1040" t="n">
@@ -46958,7 +46958,7 @@
         </is>
       </c>
       <c r="C1041" t="n">
-        <v>0</v>
+        <v>8800</v>
       </c>
       <c r="D1041" t="inlineStr">
         <is>
@@ -46967,7 +46967,7 @@
       </c>
       <c r="E1041" t="inlineStr">
         <is>
-          <t>1/3 Seite</t>
+          <t>1/3 Seite 4c</t>
         </is>
       </c>
       <c r="F1041" t="n">
@@ -47004,7 +47004,7 @@
         </is>
       </c>
       <c r="C1042" t="n">
-        <v>0</v>
+        <v>8800</v>
       </c>
       <c r="D1042" t="inlineStr">
         <is>
@@ -47013,7 +47013,7 @@
       </c>
       <c r="E1042" t="inlineStr">
         <is>
-          <t>1/4 Seite</t>
+          <t>1/4 Seite 4c</t>
         </is>
       </c>
       <c r="F1042" t="n">
@@ -47050,7 +47050,7 @@
         </is>
       </c>
       <c r="C1043" t="n">
-        <v>0</v>
+        <v>8800</v>
       </c>
       <c r="D1043" t="inlineStr">
         <is>
@@ -47096,7 +47096,7 @@
         </is>
       </c>
       <c r="C1044" t="n">
-        <v>0</v>
+        <v>8800</v>
       </c>
       <c r="D1044" t="inlineStr">
         <is>
@@ -47142,7 +47142,7 @@
         </is>
       </c>
       <c r="C1045" t="n">
-        <v>0</v>
+        <v>8800</v>
       </c>
       <c r="D1045" t="inlineStr">
         <is>
@@ -47151,7 +47151,7 @@
       </c>
       <c r="E1045" t="inlineStr">
         <is>
-          <t>gegenüber Textanfang</t>
+          <t>Seite ggü. Textanfang</t>
         </is>
       </c>
       <c r="F1045" t="n">
@@ -47188,7 +47188,7 @@
         </is>
       </c>
       <c r="C1046" t="n">
-        <v>0</v>
+        <v>8800</v>
       </c>
       <c r="D1046" t="inlineStr">
         <is>
@@ -47234,7 +47234,7 @@
         </is>
       </c>
       <c r="C1047" t="n">
-        <v>0</v>
+        <v>8800</v>
       </c>
       <c r="D1047" t="inlineStr">
         <is>
@@ -47280,7 +47280,7 @@
         </is>
       </c>
       <c r="C1048" t="n">
-        <v>0</v>
+        <v>8800</v>
       </c>
       <c r="D1048" t="inlineStr">
         <is>
@@ -47326,7 +47326,7 @@
         </is>
       </c>
       <c r="C1049" t="n">
-        <v>0</v>
+        <v>8800</v>
       </c>
       <c r="D1049" t="inlineStr">
         <is>
@@ -47372,7 +47372,7 @@
         </is>
       </c>
       <c r="C1050" t="n">
-        <v>0</v>
+        <v>8800</v>
       </c>
       <c r="D1050" t="inlineStr">
         <is>
@@ -47418,7 +47418,7 @@
         </is>
       </c>
       <c r="C1051" t="n">
-        <v>0</v>
+        <v>8800</v>
       </c>
       <c r="D1051" t="inlineStr">
         <is>
@@ -47459,7 +47459,7 @@
         </is>
       </c>
       <c r="C1052" t="n">
-        <v>0</v>
+        <v>8800</v>
       </c>
       <c r="D1052" t="inlineStr">
         <is>
@@ -47500,7 +47500,7 @@
         </is>
       </c>
       <c r="C1053" t="n">
-        <v>0</v>
+        <v>8800</v>
       </c>
       <c r="D1053" t="inlineStr">
         <is>
@@ -47541,7 +47541,7 @@
         </is>
       </c>
       <c r="C1054" t="n">
-        <v>0</v>
+        <v>8800</v>
       </c>
       <c r="D1054" t="inlineStr">
         <is>
@@ -47582,7 +47582,7 @@
         </is>
       </c>
       <c r="C1055" t="n">
-        <v>0</v>
+        <v>8800</v>
       </c>
       <c r="D1055" t="inlineStr">
         <is>
@@ -47628,7 +47628,7 @@
         </is>
       </c>
       <c r="C1056" t="n">
-        <v>0</v>
+        <v>8800</v>
       </c>
       <c r="D1056" t="inlineStr">
         <is>
@@ -47669,7 +47669,7 @@
         </is>
       </c>
       <c r="C1057" t="n">
-        <v>0</v>
+        <v>8800</v>
       </c>
       <c r="D1057" t="inlineStr">
         <is>
@@ -47710,7 +47710,7 @@
         </is>
       </c>
       <c r="C1058" t="n">
-        <v>0</v>
+        <v>8800</v>
       </c>
       <c r="D1058" t="inlineStr">
         <is>
@@ -47751,7 +47751,7 @@
         </is>
       </c>
       <c r="C1059" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1059" t="inlineStr">
         <is>
@@ -47760,7 +47760,7 @@
       </c>
       <c r="E1059" t="inlineStr">
         <is>
-          <t>1/1 Seite</t>
+          <t>1/1 Seite 4c</t>
         </is>
       </c>
       <c r="F1059" t="n">
@@ -47797,7 +47797,7 @@
         </is>
       </c>
       <c r="C1060" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1060" t="inlineStr">
         <is>
@@ -47806,7 +47806,7 @@
       </c>
       <c r="E1060" t="inlineStr">
         <is>
-          <t>1/2 Seite</t>
+          <t>1/2 Seite 4c</t>
         </is>
       </c>
       <c r="F1060" t="n">
@@ -47843,7 +47843,7 @@
         </is>
       </c>
       <c r="C1061" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1061" t="inlineStr">
         <is>
@@ -47852,7 +47852,7 @@
       </c>
       <c r="E1061" t="inlineStr">
         <is>
-          <t>1/3 Seite</t>
+          <t>1/3 Seite 4c</t>
         </is>
       </c>
       <c r="F1061" t="n">
@@ -47889,7 +47889,7 @@
         </is>
       </c>
       <c r="C1062" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1062" t="inlineStr">
         <is>
@@ -47898,7 +47898,7 @@
       </c>
       <c r="E1062" t="inlineStr">
         <is>
-          <t>1/4 Seite</t>
+          <t>1/4 Seite 4c</t>
         </is>
       </c>
       <c r="F1062" t="n">
@@ -47935,7 +47935,7 @@
         </is>
       </c>
       <c r="C1063" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1063" t="inlineStr">
         <is>
@@ -47981,7 +47981,7 @@
         </is>
       </c>
       <c r="C1064" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1064" t="inlineStr">
         <is>
@@ -48027,7 +48027,7 @@
         </is>
       </c>
       <c r="C1065" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1065" t="inlineStr">
         <is>
@@ -48036,7 +48036,7 @@
       </c>
       <c r="E1065" t="inlineStr">
         <is>
-          <t>Gegenüber Inhalt</t>
+          <t>Seite ggü. Inhalt</t>
         </is>
       </c>
       <c r="F1065" t="n">
@@ -48073,7 +48073,7 @@
         </is>
       </c>
       <c r="C1066" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1066" t="inlineStr">
         <is>
@@ -48119,7 +48119,7 @@
         </is>
       </c>
       <c r="C1067" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1067" t="inlineStr">
         <is>
@@ -48165,7 +48165,7 @@
         </is>
       </c>
       <c r="C1068" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1068" t="inlineStr">
         <is>
@@ -48211,7 +48211,7 @@
         </is>
       </c>
       <c r="C1069" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1069" t="inlineStr">
         <is>
@@ -48257,7 +48257,7 @@
         </is>
       </c>
       <c r="C1070" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1070" t="inlineStr">
         <is>
@@ -48298,7 +48298,7 @@
         </is>
       </c>
       <c r="C1071" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1071" t="inlineStr">
         <is>
@@ -48339,7 +48339,7 @@
         </is>
       </c>
       <c r="C1072" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1072" t="inlineStr">
         <is>
@@ -48380,7 +48380,7 @@
         </is>
       </c>
       <c r="C1073" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1073" t="inlineStr">
         <is>
@@ -48421,7 +48421,7 @@
         </is>
       </c>
       <c r="C1074" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1074" t="inlineStr">
         <is>
@@ -48462,7 +48462,7 @@
         </is>
       </c>
       <c r="C1075" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1075" t="inlineStr">
         <is>
@@ -48508,7 +48508,7 @@
         </is>
       </c>
       <c r="C1076" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1076" t="inlineStr">
         <is>
@@ -48549,7 +48549,7 @@
         </is>
       </c>
       <c r="C1077" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1077" t="inlineStr">
         <is>
@@ -48590,7 +48590,7 @@
         </is>
       </c>
       <c r="C1078" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D1078" t="inlineStr">
         <is>
@@ -48631,7 +48631,7 @@
         </is>
       </c>
       <c r="C1079" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="D1079" t="inlineStr">
         <is>
@@ -48640,7 +48640,7 @@
       </c>
       <c r="E1079" t="inlineStr">
         <is>
-          <t>1/1 Seite</t>
+          <t>1/1 Seite 4c</t>
         </is>
       </c>
       <c r="F1079" t="n">
@@ -48677,7 +48677,7 @@
         </is>
       </c>
       <c r="C1080" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="D1080" t="inlineStr">
         <is>
@@ -48686,7 +48686,7 @@
       </c>
       <c r="E1080" t="inlineStr">
         <is>
-          <t>1/2 Seite</t>
+          <t>1/2 Seite 4c</t>
         </is>
       </c>
       <c r="F1080" t="n">
@@ -48723,7 +48723,7 @@
         </is>
       </c>
       <c r="C1081" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="D1081" t="inlineStr">
         <is>
@@ -48732,7 +48732,7 @@
       </c>
       <c r="E1081" t="inlineStr">
         <is>
-          <t>1/3 seite</t>
+          <t>1/3 Seite 4c</t>
         </is>
       </c>
       <c r="F1081" t="n">
@@ -48769,7 +48769,7 @@
         </is>
       </c>
       <c r="C1082" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="D1082" t="inlineStr">
         <is>
@@ -48778,7 +48778,7 @@
       </c>
       <c r="E1082" t="inlineStr">
         <is>
-          <t>1/4 Seite</t>
+          <t>1/4 Seite 4c</t>
         </is>
       </c>
       <c r="F1082" t="n">
@@ -48815,7 +48815,7 @@
         </is>
       </c>
       <c r="C1083" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="D1083" t="inlineStr">
         <is>
@@ -48861,7 +48861,7 @@
         </is>
       </c>
       <c r="C1084" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="D1084" t="inlineStr">
         <is>
@@ -48907,7 +48907,7 @@
         </is>
       </c>
       <c r="C1085" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="D1085" t="inlineStr">
         <is>
@@ -48916,7 +48916,7 @@
       </c>
       <c r="E1085" t="inlineStr">
         <is>
-          <t>gegenüber Textanfang</t>
+          <t>Seite ggü. Textanfang</t>
         </is>
       </c>
       <c r="F1085" t="n">
@@ -48953,7 +48953,7 @@
         </is>
       </c>
       <c r="C1086" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="D1086" t="inlineStr">
         <is>
@@ -48999,7 +48999,7 @@
         </is>
       </c>
       <c r="C1087" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="D1087" t="inlineStr">
         <is>
@@ -49045,7 +49045,7 @@
         </is>
       </c>
       <c r="C1088" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="D1088" t="inlineStr">
         <is>
@@ -49091,7 +49091,7 @@
         </is>
       </c>
       <c r="C1089" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="D1089" t="inlineStr">
         <is>
@@ -49137,7 +49137,7 @@
         </is>
       </c>
       <c r="C1090" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="D1090" t="inlineStr">
         <is>
@@ -49183,7 +49183,7 @@
         </is>
       </c>
       <c r="C1091" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="D1091" t="inlineStr">
         <is>
@@ -49224,7 +49224,7 @@
         </is>
       </c>
       <c r="C1092" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="D1092" t="inlineStr">
         <is>
@@ -49265,7 +49265,7 @@
         </is>
       </c>
       <c r="C1093" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="D1093" t="inlineStr">
         <is>
@@ -49306,7 +49306,7 @@
         </is>
       </c>
       <c r="C1094" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="D1094" t="inlineStr">
         <is>
@@ -49347,7 +49347,7 @@
         </is>
       </c>
       <c r="C1095" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="D1095" t="inlineStr">
         <is>
@@ -49388,7 +49388,7 @@
         </is>
       </c>
       <c r="C1096" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="D1096" t="inlineStr">
         <is>
@@ -49429,7 +49429,7 @@
         </is>
       </c>
       <c r="C1097" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="D1097" t="inlineStr">
         <is>
@@ -49470,7 +49470,7 @@
         </is>
       </c>
       <c r="C1098" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="D1098" t="inlineStr">
         <is>
@@ -49516,7 +49516,7 @@
         </is>
       </c>
       <c r="C1099" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="D1099" t="inlineStr">
         <is>
@@ -49557,7 +49557,7 @@
         </is>
       </c>
       <c r="C1100" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="D1100" t="inlineStr">
         <is>
@@ -49566,7 +49566,7 @@
       </c>
       <c r="E1100" t="inlineStr">
         <is>
-          <t>1/1 Seite</t>
+          <t>1/1 Seite 4c</t>
         </is>
       </c>
       <c r="F1100" t="n">
@@ -49603,7 +49603,7 @@
         </is>
       </c>
       <c r="C1101" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="D1101" t="inlineStr">
         <is>
@@ -49612,7 +49612,7 @@
       </c>
       <c r="E1101" t="inlineStr">
         <is>
-          <t>1/2 Seite</t>
+          <t>1/2 Seite 4c</t>
         </is>
       </c>
       <c r="F1101" t="n">
@@ -49649,7 +49649,7 @@
         </is>
       </c>
       <c r="C1102" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="D1102" t="inlineStr">
         <is>
@@ -49658,7 +49658,7 @@
       </c>
       <c r="E1102" t="inlineStr">
         <is>
-          <t>1/3 Seite</t>
+          <t>1/3 Seite 4c</t>
         </is>
       </c>
       <c r="F1102" t="n">
@@ -49695,7 +49695,7 @@
         </is>
       </c>
       <c r="C1103" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="D1103" t="inlineStr">
         <is>
@@ -49704,7 +49704,7 @@
       </c>
       <c r="E1103" t="inlineStr">
         <is>
-          <t>1/4 Seite</t>
+          <t>1/4 Seite 4c</t>
         </is>
       </c>
       <c r="F1103" t="n">
@@ -49741,7 +49741,7 @@
         </is>
       </c>
       <c r="C1104" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="D1104" t="inlineStr">
         <is>
@@ -49787,7 +49787,7 @@
         </is>
       </c>
       <c r="C1105" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="D1105" t="inlineStr">
         <is>
@@ -49833,7 +49833,7 @@
         </is>
       </c>
       <c r="C1106" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="D1106" t="inlineStr">
         <is>
@@ -49842,7 +49842,7 @@
       </c>
       <c r="E1106" t="inlineStr">
         <is>
-          <t>Gegenüber Inhalt</t>
+          <t>Seite ggü. Inhalt</t>
         </is>
       </c>
       <c r="F1106" t="n">
@@ -49879,7 +49879,7 @@
         </is>
       </c>
       <c r="C1107" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="D1107" t="inlineStr">
         <is>
@@ -49925,7 +49925,7 @@
         </is>
       </c>
       <c r="C1108" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="D1108" t="inlineStr">
         <is>
@@ -49971,7 +49971,7 @@
         </is>
       </c>
       <c r="C1109" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="D1109" t="inlineStr">
         <is>
@@ -50017,7 +50017,7 @@
         </is>
       </c>
       <c r="C1110" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="D1110" t="inlineStr">
         <is>
@@ -50063,7 +50063,7 @@
         </is>
       </c>
       <c r="C1111" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="D1111" t="inlineStr">
         <is>
@@ -50104,7 +50104,7 @@
         </is>
       </c>
       <c r="C1112" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="D1112" t="inlineStr">
         <is>
@@ -50145,7 +50145,7 @@
         </is>
       </c>
       <c r="C1113" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="D1113" t="inlineStr">
         <is>
@@ -50186,7 +50186,7 @@
         </is>
       </c>
       <c r="C1114" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="D1114" t="inlineStr">
         <is>
@@ -50227,7 +50227,7 @@
         </is>
       </c>
       <c r="C1115" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="D1115" t="inlineStr">
         <is>
@@ -50273,7 +50273,7 @@
         </is>
       </c>
       <c r="C1116" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="D1116" t="inlineStr">
         <is>
@@ -50314,7 +50314,7 @@
         </is>
       </c>
       <c r="C1117" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="D1117" t="inlineStr">
         <is>
@@ -50355,7 +50355,7 @@
         </is>
       </c>
       <c r="C1118" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="D1118" t="inlineStr">
         <is>
@@ -50396,7 +50396,7 @@
         </is>
       </c>
       <c r="C1119" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="D1119" t="inlineStr">
         <is>
@@ -51260,7 +51260,7 @@
         </is>
       </c>
       <c r="C1138" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="D1138" t="inlineStr">
         <is>
@@ -51306,7 +51306,7 @@
         </is>
       </c>
       <c r="C1139" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="D1139" t="inlineStr">
         <is>
@@ -51352,7 +51352,7 @@
         </is>
       </c>
       <c r="C1140" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="D1140" t="inlineStr">
         <is>
@@ -51398,7 +51398,7 @@
         </is>
       </c>
       <c r="C1141" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="D1141" t="inlineStr">
         <is>
@@ -51444,7 +51444,7 @@
         </is>
       </c>
       <c r="C1142" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="D1142" t="inlineStr">
         <is>
@@ -51490,7 +51490,7 @@
         </is>
       </c>
       <c r="C1143" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="D1143" t="inlineStr">
         <is>
@@ -51536,7 +51536,7 @@
         </is>
       </c>
       <c r="C1144" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="D1144" t="inlineStr">
         <is>
@@ -51582,7 +51582,7 @@
         </is>
       </c>
       <c r="C1145" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="D1145" t="inlineStr">
         <is>
@@ -51628,7 +51628,7 @@
         </is>
       </c>
       <c r="C1146" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="D1146" t="inlineStr">
         <is>
@@ -51674,7 +51674,7 @@
         </is>
       </c>
       <c r="C1147" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="D1147" t="inlineStr">
         <is>
@@ -51720,7 +51720,7 @@
         </is>
       </c>
       <c r="C1148" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="D1148" t="inlineStr">
         <is>
@@ -51766,7 +51766,7 @@
         </is>
       </c>
       <c r="C1149" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="D1149" t="inlineStr">
         <is>
@@ -51812,7 +51812,7 @@
         </is>
       </c>
       <c r="C1150" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="D1150" t="inlineStr">
         <is>
@@ -51858,7 +51858,7 @@
         </is>
       </c>
       <c r="C1151" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="D1151" t="inlineStr">
         <is>
@@ -51904,7 +51904,7 @@
         </is>
       </c>
       <c r="C1152" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="D1152" t="inlineStr">
         <is>
@@ -51950,7 +51950,7 @@
         </is>
       </c>
       <c r="C1153" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="D1153" t="inlineStr">
         <is>
@@ -51996,7 +51996,7 @@
         </is>
       </c>
       <c r="C1154" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="D1154" t="inlineStr">
         <is>
@@ -72494,6 +72494,26 @@
           <t>Februar</t>
         </is>
       </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>12.02.</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>15.01.</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>19.01.</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>29.01.</t>
+        </is>
+      </c>
       <c r="I210" t="inlineStr">
         <is>
           <t>Hypertonie</t>
@@ -72519,6 +72539,26 @@
           <t>März</t>
         </is>
       </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>16.03.</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>17.02.</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>19.02.</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>02.03.</t>
+        </is>
+      </c>
       <c r="I211" t="inlineStr">
         <is>
           <t>Kardiologie</t>
@@ -72544,6 +72584,26 @@
           <t>Juni</t>
         </is>
       </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>10.06.</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>14.05.</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>18.05.</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>28.05.</t>
+        </is>
+      </c>
       <c r="I212" t="inlineStr">
         <is>
           <t>Adipositas / Diabetes</t>
@@ -72569,6 +72629,26 @@
           <t>September</t>
         </is>
       </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>17.09.</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>24.08.</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>26.08.</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>06.09.</t>
+        </is>
+      </c>
       <c r="I213" t="inlineStr">
         <is>
           <t>Kardiologie</t>
@@ -72594,6 +72674,26 @@
           <t>Oktober</t>
         </is>
       </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>22.10.</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>28.09.</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>30.09.</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>11.10.</t>
+        </is>
+      </c>
       <c r="I214" t="inlineStr">
         <is>
           <t>Neurologie</t>
@@ -72619,6 +72719,26 @@
           <t>Dezember</t>
         </is>
       </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>10.12.</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>16.11.</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>18.11.</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>29.11.</t>
+        </is>
+      </c>
       <c r="I215" t="inlineStr">
         <is>
           <t>Angiologie / Lipidologie</t>
@@ -74641,6 +74761,26 @@
           <t>Februar</t>
         </is>
       </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>26.02.</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>02.02.</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>04.02.</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>16.02.</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="n">
@@ -74661,6 +74801,26 @@
           <t>April</t>
         </is>
       </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>23.04.</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>30.03.</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>01.04.</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>13.04.</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="n">
@@ -74681,6 +74841,26 @@
           <t>Juni</t>
         </is>
       </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>25.06.</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>02.06.</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>04.06.</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>15.06.</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="n">
@@ -74701,6 +74881,26 @@
           <t>September</t>
         </is>
       </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>03.09.</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>11.08.</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>13.08.</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>24.08.</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="n">
@@ -74721,6 +74921,26 @@
           <t>Oktober</t>
         </is>
       </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>28.10.</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>05.10.</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>07.10.</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>18.10.</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="n">
@@ -74741,6 +74961,26 @@
           <t>Dezember</t>
         </is>
       </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>10.12.</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>17.11.</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>19.11.</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>30.11.</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="n">
@@ -74761,6 +75001,21 @@
           <t>Februar</t>
         </is>
       </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>12.02.</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>25.01.</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>29.01.</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -74781,6 +75036,21 @@
           <t>März</t>
         </is>
       </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>12.03.</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>22.02.</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>26.02.</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="n">
@@ -74801,6 +75071,21 @@
           <t>April</t>
         </is>
       </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>23.04.</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>05.04.</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>09.04.</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -74821,6 +75106,21 @@
           <t>Mai</t>
         </is>
       </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>21.05.</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>29.04.</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>05.05.</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="n">
@@ -74841,6 +75141,21 @@
           <t>Juni</t>
         </is>
       </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>25.06.</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>04.06.</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>10.06.</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="n">
@@ -74861,6 +75176,21 @@
           <t>August</t>
         </is>
       </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>13.08.</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>26.07.</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>30.07.</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="n">
@@ -74881,6 +75211,21 @@
           <t>September</t>
         </is>
       </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>24.09.</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>06.09.</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>10.09.</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="n">
@@ -74901,6 +75246,21 @@
           <t>Oktober</t>
         </is>
       </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>29.10.</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>11.10.</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>15.10.</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="n">
@@ -74919,6 +75279,21 @@
       <c r="D280" t="inlineStr">
         <is>
           <t>Dezember</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>10.12.</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>22.11.</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>26.11.</t>
         </is>
       </c>
     </row>

</xml_diff>